<commit_message>
interpolation and extrapolation of great lakes TWL and plotting and analysis of levels.
</commit_message>
<xml_diff>
--- a/examples/great_lakes/templates/template_twl.xlsx
+++ b/examples/great_lakes/templates/template_twl.xlsx
@@ -185,6 +185,16 @@
         <t>(Optional) comma-separated explicit colorbar ticks, e.g. "-1.0, 0.0, 1.0".</t>
       </text>
     </comment>
+    <comment ref="A9" authorId="0" shapeId="0">
+      <text>
+        <t>If true, also write a second grid csv + plot png per row: the water level under every scenario equivalent (same ARI) to the baseline (_0_0) scenario's ARI at magnitude_value. See CONTEXT.md's "Equivalent elevation" definition.</t>
+      </text>
+    </comment>
+    <comment ref="A10" authorId="0" shapeId="0">
+      <text>
+        <t>If true, estimate missing (NaN) grid cells in the response surface via Delaunay triangulation before plotting (climate-canvas's --fillin option). Applies to every plot png this row produces.</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -639,7 +649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -729,6 +739,26 @@
         </is>
       </c>
       <c r="B8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>compute_equivalent_elevation</t>
+        </is>
+      </c>
+      <c r="B9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>fillin</t>
+        </is>
+      </c>
+      <c r="B10" t="b">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
longtail point runs and data
</commit_message>
<xml_diff>
--- a/examples/great_lakes/templates/template_twl.xlsx
+++ b/examples/great_lakes/templates/template_twl.xlsx
@@ -140,6 +140,11 @@
         <t>Climate-canvas plot reference line, in the config sheet's metric_mode units (portion 0-1, percentage 0-100, or return_period in years) -- NOT a water level.</t>
       </text>
     </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>Blank = skip. "baseline_magnitude" = run using this row's magnitude_value. A number = run using that water-level value instead of magnitude_value (for this analysis only).</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -186,11 +191,6 @@
       </text>
     </comment>
     <comment ref="A9" authorId="0" shapeId="0">
-      <text>
-        <t>If true, also write a second grid csv + plot png per row: the water level under every scenario equivalent (same ARI) to the baseline (_0_0) scenario's ARI at magnitude_value. See CONTEXT.md's "Equivalent elevation" definition.</t>
-      </text>
-    </comment>
-    <comment ref="A10" authorId="0" shapeId="0">
       <text>
         <t>If true, estimate missing (NaN) grid cells in the response surface via Delaunay triangulation before plotting (climate-canvas's --fillin option). Applies to every plot png this row produces.</t>
       </text>
@@ -488,7 +488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -542,6 +542,11 @@
           <t>threshold</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>equivalent_elevation</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -605,6 +610,11 @@
       <c r="I3" t="n">
         <v>176</v>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>baseline_magnitude</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -635,6 +645,9 @@
       </c>
       <c r="I4" t="n">
         <v>74.8</v>
+      </c>
+      <c r="K4" t="n">
+        <v>75.5</v>
       </c>
     </row>
   </sheetData>
@@ -649,7 +662,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -743,20 +756,10 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>compute_equivalent_elevation</t>
+          <t>fillin</t>
         </is>
       </c>
       <c r="B9" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>fillin</t>
-        </is>
-      </c>
-      <c r="B10" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>